<commit_message>
More Matt homework problems
</commit_message>
<xml_diff>
--- a/StudentGuideModule2/M_problems/potential/scratch_work_for_hard_problem_with_three_charges.xlsx
+++ b/StudentGuideModule2/M_problems/potential/scratch_work_for_hard_problem_with_three_charges.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mtrawick\Box\github\132\StudentGuideModule2\M_problems\potential\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6126AC12-F33A-4433-B585-72FE266E0017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FC04BD6-5636-45FB-86A2-4BDCADAD6378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{F161C81F-7CE3-4023-9446-1B336071E562}"/>
+    <workbookView xWindow="-240" yWindow="-240" windowWidth="38880" windowHeight="21360" xr2:uid="{F161C81F-7CE3-4023-9446-1B336071E562}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Q1</t>
   </si>
@@ -77,9 +77,6 @@
     <t xml:space="preserve">Equilibrium </t>
   </si>
   <si>
-    <t>V at x=+4</t>
-  </si>
-  <si>
     <t>V_tot at eq</t>
   </si>
   <si>
@@ -90,6 +87,18 @@
   </si>
   <si>
     <t>r at eq</t>
+  </si>
+  <si>
+    <t>V at x=eq</t>
+  </si>
+  <si>
+    <t>Vi - Vf</t>
+  </si>
+  <si>
+    <t>q(Vi-Vf)</t>
+  </si>
+  <si>
+    <t>9458 m/s</t>
   </si>
 </sst>
 </file>
@@ -97,7 +106,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0000E+00"/>
+    <numFmt numFmtId="164" formatCode="0.0000E+00"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -130,7 +139,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,16 +474,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CC01A17-D609-446A-8362-0E04E1E13141}">
-  <dimension ref="A2:D19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:D25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12.41796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="14.15625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.68359375" style="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -485,7 +494,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -496,7 +505,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -510,15 +519,15 @@
         <v>1.67E-9</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="1">
-        <v>2.8E-11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>2.8000000000000001E-14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -529,7 +538,7 @@
         <v>9000000000</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -542,7 +551,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -551,7 +560,7 @@
         <v>3750</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -560,7 +569,7 @@
         <v>6.2624999999999998E-6</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -568,9 +577,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13" s="1">
         <v>0.18</v>
@@ -579,9 +588,9 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B14" s="1">
         <f>B6*B4/B13</f>
@@ -592,40 +601,63 @@
         <v>750</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="1">
         <f>B14+C14</f>
         <v>3000</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D16" s="1">
         <f>B15*D4</f>
         <v>5.0100000000000003E-6</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D18" s="1">
         <f>D10-D16</f>
         <v>1.2524999999999994E-6</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>10</v>
       </c>
       <c r="D19" s="1">
         <f>SQRT(2*D18/D5)</f>
-        <v>299.10581023157283</v>
+        <v>9458.5562172186546</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="1">
+        <f>B9-B15</f>
+        <v>750</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="1">
+        <f>B20*D4</f>
+        <v>1.2525000000000001E-6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="D25" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>